<commit_message>
[ADD] logica de pdf + masivo
</commit_message>
<xml_diff>
--- a/Plantilla_DESEMBARGO.xlsx
+++ b/Plantilla_DESEMBARGO.xlsx
@@ -1,16 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="5"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Documents\Trabajo\JT\back-jt\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEAAF690-79C3-445D-BCE9-8FE3C8053A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="DESEMBARGO" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="DESEMBARGO" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -22,98 +27,95 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="28">
   <si>
-    <t xml:space="preserve">NO ID DEMANDADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO DE PROCESO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE OFICIO INICIAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE OFICIO FINAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NO. DE RADICADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO ID DEMANDADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOMBRE DEMANDADO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OFICIO DE EMBARGO A DESEMBARGAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RADICADO OFICIO DE EMBARGO A DESEMBARGAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIPO DOCUMENTO RECIBIDO EN EMAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">214321013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JUDICIAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prueba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20250232006224 DEL 241125 00000000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1128</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KEVINCITO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">68001400300520240075800</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1129</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KEVINCITO 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">68001400300520240075801</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KEVINCITO 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">68001400300520240075802</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COACTIVO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SERGIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">68001400300520240075803</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SERGIO 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">68001400300520240075804</t>
+    <t>NO ID DEMANDADO</t>
+  </si>
+  <si>
+    <t>TIPO DE PROCESO</t>
+  </si>
+  <si>
+    <t>NOMBRE OFICIO INICIAL</t>
+  </si>
+  <si>
+    <t>NOMBRE OFICIO FINAL</t>
+  </si>
+  <si>
+    <t>NO. DE RADICADO</t>
+  </si>
+  <si>
+    <t>TIPO ID DEMANDADO</t>
+  </si>
+  <si>
+    <t>NOMBRE DEMANDADO</t>
+  </si>
+  <si>
+    <t>OFICIO DE EMBARGO A DESEMBARGAR</t>
+  </si>
+  <si>
+    <t>RADICADO OFICIO DE EMBARGO A DESEMBARGAR</t>
+  </si>
+  <si>
+    <t>TIPO DOCUMENTO RECIBIDO EN EMAIL</t>
+  </si>
+  <si>
+    <t>214321013</t>
+  </si>
+  <si>
+    <t>JUDICIAL</t>
+  </si>
+  <si>
+    <t>Prueba</t>
+  </si>
+  <si>
+    <t>20250232006224 DEL 241125 00000000</t>
+  </si>
+  <si>
+    <t>1128</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>KEVINCITO</t>
+  </si>
+  <si>
+    <t>68001400300520240075800</t>
+  </si>
+  <si>
+    <t>1129</t>
+  </si>
+  <si>
+    <t>KEVINCITO 1</t>
+  </si>
+  <si>
+    <t>68001400300520240075801</t>
+  </si>
+  <si>
+    <t>KEVINCITO 2</t>
+  </si>
+  <si>
+    <t>68001400300520240075802</t>
+  </si>
+  <si>
+    <t>COACTIVO</t>
+  </si>
+  <si>
+    <t>SERGIO</t>
+  </si>
+  <si>
+    <t>68001400300520240075803</t>
+  </si>
+  <si>
+    <t>SERGIO 2</t>
+  </si>
+  <si>
+    <t>68001400300520240075804</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,26 +124,10 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -160,68 +146,44 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -280,13 +242,29 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF2F5496"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -328,12 +306,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -362,7 +340,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -380,7 +358,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -431,7 +409,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -449,34 +427,33 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="33.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="36"/>
+    <col min="1" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="33.88671875" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="35" customWidth="1"/>
+    <col min="9" max="9" width="44" customWidth="1"/>
+    <col min="10" max="10" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -508,7 +485,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -536,11 +513,11 @@
       <c r="I2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -568,11 +545,11 @@
       <c r="I3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="J3" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -600,11 +577,11 @@
       <c r="I4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -632,11 +609,11 @@
       <c r="I5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -664,20 +641,15 @@
       <c r="I6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C7" s="2"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>